<commit_message>
align to the right and bold font implemented
</commit_message>
<xml_diff>
--- a/tabela.xlsx
+++ b/tabela.xlsx
@@ -11,7 +11,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <name val="Calibri"/>
@@ -19,6 +19,11 @@
     <font>
       <sz val="12"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,10 +57,14 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -390,352 +399,352 @@
   <dimension ref="A1:D25"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="str">
+      <c r="A1" s="3" t="str">
         <v>Godzina</v>
       </c>
-      <c r="B1" s="2" t="str">
+      <c r="B1" s="3" t="str">
         <v>01-01-2025</v>
       </c>
-      <c r="C1" s="2" t="str">
+      <c r="C1" s="3" t="str">
         <v>02-01-2025</v>
       </c>
-      <c r="D1" s="2" t="str">
+      <c r="D1" s="3" t="str">
         <v>03-01-2025</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="3" t="str">
         <v>0:00</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>-20,00</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>-64,50</v>
       </c>
-      <c r="D2" s="2" t="str">
+      <c r="D2" s="4" t="str">
         <v>367,06</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="3" t="str">
         <v>1:00</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>-20,00</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="4" t="str">
         <v>-45,01</v>
       </c>
-      <c r="D3" s="2" t="str">
+      <c r="D3" s="4" t="str">
         <v>321,20</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="str">
+      <c r="A4" s="3" t="str">
         <v>2:00</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="4" t="str">
         <v>-35,00</v>
       </c>
-      <c r="C4" s="2" t="str">
+      <c r="C4" s="4" t="str">
         <v>-45,01</v>
       </c>
-      <c r="D4" s="2" t="str">
+      <c r="D4" s="4" t="str">
         <v>295,39</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="str">
+      <c r="A5" s="3" t="str">
         <v>3:00</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="4" t="str">
         <v>-50,00</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="4" t="str">
         <v>-45,01</v>
       </c>
-      <c r="D5" s="2" t="str">
+      <c r="D5" s="4" t="str">
         <v>280,00</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="str">
+      <c r="A6" s="3" t="str">
         <v>4:00</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B6" s="4" t="str">
         <v>-76,40</v>
       </c>
-      <c r="C6" s="2" t="str">
+      <c r="C6" s="4" t="str">
         <v>-49,99</v>
       </c>
-      <c r="D6" s="2" t="str">
+      <c r="D6" s="4" t="str">
         <v>279,99</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="str">
+      <c r="A7" s="3" t="str">
         <v>5:00</v>
       </c>
-      <c r="B7" s="2" t="str">
+      <c r="B7" s="4" t="str">
         <v>-73,06</v>
       </c>
-      <c r="C7" s="2" t="str">
+      <c r="C7" s="4" t="str">
         <v>-4,12</v>
       </c>
-      <c r="D7" s="2" t="str">
+      <c r="D7" s="4" t="str">
         <v>317,80</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="str">
+      <c r="A8" s="3" t="str">
         <v>6:00</v>
       </c>
-      <c r="B8" s="2" t="str">
+      <c r="B8" s="4" t="str">
         <v>-130,00</v>
       </c>
-      <c r="C8" s="2" t="str">
+      <c r="C8" s="4" t="str">
         <v>127,99</v>
       </c>
-      <c r="D8" s="2" t="str">
+      <c r="D8" s="4" t="str">
         <v>427,00</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="str">
+      <c r="A9" s="3" t="str">
         <v>7:00</v>
       </c>
-      <c r="B9" s="2" t="str">
+      <c r="B9" s="4" t="str">
         <v>-150,00</v>
       </c>
-      <c r="C9" s="2" t="str">
+      <c r="C9" s="4" t="str">
         <v>329,99</v>
       </c>
-      <c r="D9" s="2" t="str">
+      <c r="D9" s="4" t="str">
         <v>442,00</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="str">
+      <c r="A10" s="3" t="str">
         <v>8:00</v>
       </c>
-      <c r="B10" s="2" t="str">
+      <c r="B10" s="4" t="str">
         <v>-200,00</v>
       </c>
-      <c r="C10" s="2" t="str">
+      <c r="C10" s="4" t="str">
         <v>384,99</v>
       </c>
-      <c r="D10" s="2" t="str">
+      <c r="D10" s="4" t="str">
         <v>482,00</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="str">
+      <c r="A11" s="3" t="str">
         <v>9:00</v>
       </c>
-      <c r="B11" s="2" t="str">
+      <c r="B11" s="4" t="str">
         <v>-264,00</v>
       </c>
-      <c r="C11" s="2" t="str">
+      <c r="C11" s="4" t="str">
         <v>401,38</v>
       </c>
-      <c r="D11" s="2" t="str">
+      <c r="D11" s="4" t="str">
         <v>463,25</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="str">
+      <c r="A12" s="3" t="str">
         <v>10:00</v>
       </c>
-      <c r="B12" s="2" t="str">
+      <c r="B12" s="4" t="str">
         <v>-265,00</v>
       </c>
-      <c r="C12" s="2" t="str">
+      <c r="C12" s="4" t="str">
         <v>384,99</v>
       </c>
-      <c r="D12" s="2" t="str">
+      <c r="D12" s="4" t="str">
         <v>394,00</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="str">
+      <c r="A13" s="3" t="str">
         <v>11:00</v>
       </c>
-      <c r="B13" s="2" t="str">
+      <c r="B13" s="4" t="str">
         <v>-265,00</v>
       </c>
-      <c r="C13" s="2" t="str">
+      <c r="C13" s="4" t="str">
         <v>386,30</v>
       </c>
-      <c r="D13" s="2" t="str">
+      <c r="D13" s="4" t="str">
         <v>360,00</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="str">
+      <c r="A14" s="3" t="str">
         <v>12:00</v>
       </c>
-      <c r="B14" s="2" t="str">
+      <c r="B14" s="4" t="str">
         <v>-200,00</v>
       </c>
-      <c r="C14" s="2" t="str">
+      <c r="C14" s="4" t="str">
         <v>384,99</v>
       </c>
-      <c r="D14" s="2" t="str">
+      <c r="D14" s="4" t="str">
         <v>356,23</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="str">
+      <c r="A15" s="3" t="str">
         <v>13:00</v>
       </c>
-      <c r="B15" s="2" t="str">
+      <c r="B15" s="4" t="str">
         <v>-60,01</v>
       </c>
-      <c r="C15" s="2" t="str">
+      <c r="C15" s="4" t="str">
         <v>418,60</v>
       </c>
-      <c r="D15" s="2" t="str">
+      <c r="D15" s="4" t="str">
         <v>365,11</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="str">
+      <c r="A16" s="3" t="str">
         <v>14:00</v>
       </c>
-      <c r="B16" s="2" t="str">
+      <c r="B16" s="4" t="str">
         <v>-28,80</v>
       </c>
-      <c r="C16" s="2" t="str">
+      <c r="C16" s="4" t="str">
         <v>451,03</v>
       </c>
-      <c r="D16" s="2" t="str">
+      <c r="D16" s="4" t="str">
         <v>394,00</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="str">
+      <c r="A17" s="3" t="str">
         <v>15:00</v>
       </c>
-      <c r="B17" s="2" t="str">
+      <c r="B17" s="4" t="str">
         <v>-4,12</v>
       </c>
-      <c r="C17" s="2" t="str">
+      <c r="C17" s="4" t="str">
         <v>517,52</v>
       </c>
-      <c r="D17" s="2" t="str">
+      <c r="D17" s="4" t="str">
         <v>440,00</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="str">
+      <c r="A18" s="3" t="str">
         <v>16:00</v>
       </c>
-      <c r="B18" s="2" t="str">
+      <c r="B18" s="4" t="str">
         <v>0,01</v>
       </c>
-      <c r="C18" s="2" t="str">
+      <c r="C18" s="4" t="str">
         <v>555,36</v>
       </c>
-      <c r="D18" s="2" t="str">
+      <c r="D18" s="4" t="str">
         <v>475,00</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="str">
+      <c r="A19" s="3" t="str">
         <v>17:00</v>
       </c>
-      <c r="B19" s="2" t="str">
+      <c r="B19" s="4" t="str">
         <v>0,02</v>
       </c>
-      <c r="C19" s="2" t="str">
+      <c r="C19" s="4" t="str">
         <v>576,90</v>
       </c>
-      <c r="D19" s="2" t="str">
+      <c r="D19" s="4" t="str">
         <v>480,00</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="str">
+      <c r="A20" s="3" t="str">
         <v>18:00</v>
       </c>
-      <c r="B20" s="2" t="str">
+      <c r="B20" s="4" t="str">
         <v>5,00</v>
       </c>
-      <c r="C20" s="2" t="str">
+      <c r="C20" s="4" t="str">
         <v>585,60</v>
       </c>
-      <c r="D20" s="2" t="str">
+      <c r="D20" s="4" t="str">
         <v>481,00</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="str">
+      <c r="A21" s="3" t="str">
         <v>19:00</v>
       </c>
-      <c r="B21" s="2" t="str">
+      <c r="B21" s="4" t="str">
         <v>0,01</v>
       </c>
-      <c r="C21" s="2" t="str">
+      <c r="C21" s="4" t="str">
         <v>541,82</v>
       </c>
-      <c r="D21" s="2" t="str">
+      <c r="D21" s="4" t="str">
         <v>480,00</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="str">
+      <c r="A22" s="3" t="str">
         <v>20:00</v>
       </c>
-      <c r="B22" s="2" t="str">
+      <c r="B22" s="4" t="str">
         <v>0,01</v>
       </c>
-      <c r="C22" s="2" t="str">
+      <c r="C22" s="4" t="str">
         <v>520,00</v>
       </c>
-      <c r="D22" s="2" t="str">
+      <c r="D22" s="4" t="str">
         <v>442,90</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="str">
+      <c r="A23" s="3" t="str">
         <v>21:00</v>
       </c>
-      <c r="B23" s="2" t="str">
+      <c r="B23" s="4" t="str">
         <v>-1,10</v>
       </c>
-      <c r="C23" s="2" t="str">
+      <c r="C23" s="4" t="str">
         <v>457,67</v>
       </c>
-      <c r="D23" s="2" t="str">
+      <c r="D23" s="4" t="str">
         <v>380,00</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="str">
+      <c r="A24" s="3" t="str">
         <v>22:00</v>
       </c>
-      <c r="B24" s="2" t="str">
+      <c r="B24" s="4" t="str">
         <v>-1,60</v>
       </c>
-      <c r="C24" s="2" t="str">
+      <c r="C24" s="4" t="str">
         <v>440,00</v>
       </c>
-      <c r="D24" s="2" t="str">
+      <c r="D24" s="4" t="str">
         <v>380,00</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="str">
+      <c r="A25" s="3" t="str">
         <v>23:00</v>
       </c>
-      <c r="B25" s="2" t="str">
+      <c r="B25" s="4" t="str">
         <v>-35,00</v>
       </c>
-      <c r="C25" s="2" t="str">
+      <c r="C25" s="4" t="str">
         <v>357,15</v>
       </c>
-      <c r="D25" s="2" t="str">
+      <c r="D25" s="4" t="str">
         <v>298,43</v>
       </c>
     </row>

</xml_diff>